<commit_message>
Update data files and LaTeX documents for the investigation on hydrogen peroxide decomposition. Modified binary data files, updated LaTeX source with new uncertainty calculations, and adjusted figures. Removed outdated log files and temporary sync files.
</commit_message>
<xml_diff>
--- a/Data/.xlsx
+++ b/Data/.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wrca-my.sharepoint.com/personal/huj26_mywrca_ca/Documents/12/Chemistry HL/Chemistry IA/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3273" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A5A52CE-C296-D646-BB60-323A6380752C}"/>
+  <xr:revisionPtr revIDLastSave="3342" documentId="8_{ED69E5BD-9A97-5849-9651-1A764BC4410F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF6163CA-60BF-9C4A-89DC-FB484AD5578F}"/>
   <bookViews>
-    <workbookView xWindow="-36000" yWindow="16120" windowWidth="36000" windowHeight="22500" activeTab="1" xr2:uid="{3196E468-6A35-EA40-9409-42F714E37880}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{3196E468-6A35-EA40-9409-42F714E37880}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -39,8 +39,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="74">
   <si>
     <t>Target (°C)</t>
   </si>
@@ -291,6 +313,18 @@
   <si>
     <t>Arrhenius Uncertainties</t>
   </si>
+  <si>
+    <t>arrhenius x</t>
+  </si>
+  <si>
+    <t>arrhenius y</t>
+  </si>
+  <si>
+    <t>arrhenius slope</t>
+  </si>
+  <si>
+    <t>arrhenius slope uncertainty</t>
+  </si>
 </sst>
 </file>
 
@@ -423,7 +457,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="69">
+  <borders count="74">
     <border>
       <left/>
       <right/>
@@ -1301,11 +1335,62 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="276">
+  <cellXfs count="289">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2132,6 +2217,45 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="6" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="6" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="6" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="6" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2351,28 +2475,28 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="40"/>
                   <c:pt idx="0">
-                    <c:v>1.7596985360013531E-7</c:v>
+                    <c:v>1.6814897121790712E-7</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>4.4370293644599947E-7</c:v>
+                    <c:v>4.2398280593728841E-7</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.8822893176888274E-7</c:v>
+                    <c:v>2.7541875702359903E-7</c:v>
                   </c:pt>
                   <c:pt idx="15">
-                    <c:v>1.1955215397196222E-6</c:v>
+                    <c:v>1.1423872490654169E-6</c:v>
                   </c:pt>
                   <c:pt idx="20">
-                    <c:v>9.2923209561911543E-7</c:v>
+                    <c:v>8.8793289136937687E-7</c:v>
                   </c:pt>
                   <c:pt idx="25">
-                    <c:v>1.2117876573322692E-6</c:v>
+                    <c:v>1.1579304281175019E-6</c:v>
                   </c:pt>
                   <c:pt idx="30">
-                    <c:v>2.711288692750651E-6</c:v>
+                    <c:v>2.5907869730728439E-6</c:v>
                   </c:pt>
                   <c:pt idx="35">
-                    <c:v>3.820488923827413E-6</c:v>
+                    <c:v>3.6506894161017504E-6</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -2384,28 +2508,28 @@
                   <c:formatCode>General</c:formatCode>
                   <c:ptCount val="40"/>
                   <c:pt idx="0">
-                    <c:v>1.7596985360013531E-7</c:v>
+                    <c:v>1.6814897121790712E-7</c:v>
                   </c:pt>
                   <c:pt idx="5">
-                    <c:v>4.4370293644599947E-7</c:v>
+                    <c:v>4.2398280593728841E-7</c:v>
                   </c:pt>
                   <c:pt idx="10">
-                    <c:v>2.8822893176888274E-7</c:v>
+                    <c:v>2.7541875702359903E-7</c:v>
                   </c:pt>
                   <c:pt idx="15">
-                    <c:v>1.1955215397196222E-6</c:v>
+                    <c:v>1.1423872490654169E-6</c:v>
                   </c:pt>
                   <c:pt idx="20">
-                    <c:v>9.2923209561911543E-7</c:v>
+                    <c:v>8.8793289136937687E-7</c:v>
                   </c:pt>
                   <c:pt idx="25">
-                    <c:v>1.2117876573322692E-6</c:v>
+                    <c:v>1.1579304281175019E-6</c:v>
                   </c:pt>
                   <c:pt idx="30">
-                    <c:v>2.711288692750651E-6</c:v>
+                    <c:v>2.5907869730728439E-6</c:v>
                   </c:pt>
                   <c:pt idx="35">
-                    <c:v>3.820488923827413E-6</c:v>
+                    <c:v>3.6506894161017504E-6</c:v>
                   </c:pt>
                 </c:numCache>
               </c:numRef>
@@ -2560,28 +2684,28 @@
                 <c:formatCode>0.000E+00</c:formatCode>
                 <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>1.6489947683150986E-7</c:v>
+                  <c:v>1.5757061119455391E-7</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4.4196755738981199E-7</c:v>
+                  <c:v>4.2232455483915373E-7</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2.8496029307747946E-7</c:v>
+                  <c:v>2.7229539116292476E-7</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1.1928944000136995E-6</c:v>
+                  <c:v>1.1398768711242019E-6</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>9.2616602094664455E-7</c:v>
+                  <c:v>8.8500308668234917E-7</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>1.2081347586731623E-6</c:v>
+                  <c:v>1.1544398805099108E-6</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2.7092205631905007E-6</c:v>
+                  <c:v>2.5888107603820336E-6</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>3.8173859957856402E-6</c:v>
+                  <c:v>3.6477243959729456E-6</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2734,6 +2858,7 @@
         <c:axId val="673616560"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="7.9999999999999996E-6"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -2814,7 +2939,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000E+00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.0E+00" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2854,6 +2979,7 @@
         <c:crossAx val="673811088"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
+        <c:majorUnit val="4.9999999999999998E-7"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -3716,7 +3842,7 @@
                 <a:lstStyle/>
                 <a:p>
                   <a:pPr>
-                    <a:defRPr sz="1050" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
                         <a:schemeClr val="tx1">
                           <a:lumMod val="65000"/>
@@ -8178,6 +8304,26 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{44479CEA-339A-AB42-A3E4-211097478F56}">
+  <we:reference id="wa200009404" version="1.0.0.8" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DFD131A-068C-8045-AE76-58186661ABFD}">
   <sheetPr codeName="Sheet1"/>
@@ -9874,13 +10020,13 @@
       <c r="F2" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G2" s="103" t="s">
+      <c r="G2" s="20" t="s">
         <v>16</v>
       </c>
       <c r="H2" s="116" t="s">
         <v>51</v>
       </c>
-      <c r="I2" s="106" t="s">
+      <c r="I2" s="9" t="s">
         <v>17</v>
       </c>
       <c r="J2" s="4" t="s">
@@ -9945,14 +10091,14 @@
         <f>E3+273.15</f>
         <v>287.89999999999998</v>
       </c>
-      <c r="G3" s="112">
+      <c r="G3" s="276">
         <v>25</v>
       </c>
       <c r="H3" s="152">
-        <f>(250-G3)*0.000001</f>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I3" s="113">
+        <f>(250-G3-10)*0.000001</f>
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I3" s="284">
         <v>0.3</v>
       </c>
       <c r="J3" s="110">
@@ -9973,11 +10119,11 @@
       </c>
       <c r="O3" s="153">
         <f>(H3*M3)/(8.31*D3)</f>
-        <v>1.3967665818668511E-6</v>
+        <v>1.3346880671172132E-6</v>
       </c>
       <c r="P3" s="219">
         <f>AVERAGE(O3:O7)</f>
-        <v>1.8865631315524851E-6</v>
+        <v>1.8027158812612639E-6</v>
       </c>
       <c r="Q3" s="222">
         <f>AVERAGE(M3:M7)</f>
@@ -9989,15 +10135,15 @@
       </c>
       <c r="S3" s="222">
         <f>SQRT(T3^2+((SQRT((0.5/D3)^2+(R3/Q3)^2+(0.06/225)^2))*P3)^2)</f>
-        <v>1.7596985360013531E-7</v>
+        <v>1.6814897121790712E-7</v>
       </c>
       <c r="T3" s="221">
         <f>U3/SQRT(5)</f>
-        <v>1.6489947683150986E-7</v>
+        <v>1.5757061119455391E-7</v>
       </c>
       <c r="U3" s="227">
         <f>_xlfn.STDEV.S(O3:O7)</f>
-        <v>3.6872643964940771E-7</v>
+        <v>3.5233859788721189E-7</v>
       </c>
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.2">
@@ -10019,14 +10165,14 @@
         <f t="shared" ref="F4:F42" si="1">E4+273.15</f>
         <v>288.84999999999997</v>
       </c>
-      <c r="G4" s="100">
+      <c r="G4" s="277">
         <v>25</v>
       </c>
-      <c r="H4" s="117">
-        <f t="shared" ref="H4:H42" si="2">(250-G4)*0.000001</f>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I4" s="107">
+      <c r="H4" s="281">
+        <f t="shared" ref="H4:H42" si="2">(250-G4-10)*0.000001</f>
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I4" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J4" s="27">
@@ -10047,7 +10193,7 @@
       </c>
       <c r="O4" s="145">
         <f>(H4*M4)/(8.31*D4)</f>
-        <v>1.9389458178295975E-6</v>
+        <v>1.8527704481482818E-6</v>
       </c>
       <c r="P4" s="218"/>
       <c r="Q4" s="223"/>
@@ -10075,14 +10221,14 @@
         <f t="shared" si="1"/>
         <v>287.5</v>
       </c>
-      <c r="G5" s="100">
+      <c r="G5" s="277">
         <v>25</v>
       </c>
-      <c r="H5" s="117">
+      <c r="H5" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I5" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I5" s="285">
         <v>0.32</v>
       </c>
       <c r="J5" s="27">
@@ -10103,7 +10249,7 @@
       </c>
       <c r="O5" s="145">
         <f t="shared" ref="O5:O42" si="4">(H5*M5)/(8.31*D5)</f>
-        <v>2.4117502980234296E-6</v>
+        <v>2.3045613958890553E-6</v>
       </c>
       <c r="P5" s="218"/>
       <c r="Q5" s="223"/>
@@ -10131,14 +10277,14 @@
         <f t="shared" si="1"/>
         <v>288.25</v>
       </c>
-      <c r="G6" s="100">
+      <c r="G6" s="277">
         <v>25</v>
       </c>
-      <c r="H6" s="117">
+      <c r="H6" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I6" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I6" s="285">
         <v>0.32</v>
       </c>
       <c r="J6" s="27">
@@ -10159,7 +10305,7 @@
       </c>
       <c r="O6" s="145">
         <f t="shared" si="4"/>
-        <v>1.9464033017443261E-6</v>
+        <v>1.8598964883334673E-6</v>
       </c>
       <c r="P6" s="218"/>
       <c r="Q6" s="223"/>
@@ -10176,25 +10322,25 @@
       <c r="C7" s="154">
         <v>15</v>
       </c>
-      <c r="D7" s="54">
+      <c r="D7" s="63">
         <f t="shared" si="0"/>
         <v>288.14999999999998</v>
       </c>
       <c r="E7" s="141">
         <v>14.86</v>
       </c>
-      <c r="F7" s="275">
+      <c r="F7" s="283">
         <f t="shared" si="1"/>
         <v>288.01</v>
       </c>
-      <c r="G7" s="142">
+      <c r="G7" s="278">
         <v>25</v>
       </c>
-      <c r="H7" s="155">
+      <c r="H7" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I7" s="143">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I7" s="286">
         <v>0.31</v>
       </c>
       <c r="J7" s="144">
@@ -10215,7 +10361,7 @@
       </c>
       <c r="O7" s="156">
         <f t="shared" si="4"/>
-        <v>1.7389496582982224E-6</v>
+        <v>1.6616630068183016E-6</v>
       </c>
       <c r="P7" s="220"/>
       <c r="Q7" s="224"/>
@@ -10225,59 +10371,59 @@
       <c r="U7" s="229"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A8" s="198">
+      <c r="A8" s="226">
         <v>2</v>
       </c>
-      <c r="B8" s="148">
+      <c r="B8" s="129">
         <v>1</v>
       </c>
-      <c r="C8" s="149">
+      <c r="C8" s="138">
         <v>20</v>
       </c>
-      <c r="D8" s="159">
+      <c r="D8" s="52">
         <f>C8+273.15</f>
         <v>293.14999999999998</v>
       </c>
-      <c r="E8" s="135">
+      <c r="E8" s="134">
         <v>19</v>
       </c>
       <c r="F8" s="182">
         <f t="shared" si="1"/>
         <v>292.14999999999998</v>
       </c>
-      <c r="G8" s="100">
+      <c r="G8" s="276">
         <v>25</v>
       </c>
-      <c r="H8" s="117">
+      <c r="H8" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I8" s="119">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I8" s="284">
         <v>0.3</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="110">
         <v>31.8</v>
       </c>
-      <c r="K8" s="19">
+      <c r="K8" s="111">
         <v>60</v>
       </c>
-      <c r="L8" s="150">
+      <c r="L8" s="120">
         <v>5.0999999999999997E-2</v>
       </c>
-      <c r="M8" s="19">
+      <c r="M8" s="111">
         <f t="shared" si="3"/>
         <v>1.8085106382978722</v>
       </c>
-      <c r="N8" s="186">
+      <c r="N8" s="170">
         <v>0.372</v>
       </c>
-      <c r="O8" s="151">
+      <c r="O8" s="153">
         <f t="shared" si="4"/>
-        <v>1.6703699313918148E-7</v>
-      </c>
-      <c r="P8" s="218">
+        <v>1.5961312677744008E-7</v>
+      </c>
+      <c r="P8" s="219">
         <f t="shared" ref="P8" si="5">AVERAGE(O8:O12)</f>
-        <v>1.8850179159692152E-6</v>
+        <v>1.8012393419261391E-6</v>
       </c>
       <c r="Q8" s="222">
         <f t="shared" ref="Q8" si="6">AVERAGE(M8:M12)</f>
@@ -10289,15 +10435,15 @@
       </c>
       <c r="S8" s="222">
         <f t="shared" ref="S8" si="8">SQRT(T8^2+((SQRT((0.5/D8)^2+(R8/Q8)^2+(0.06/225)^2))*P8)^2)</f>
-        <v>4.4370293644599947E-7</v>
-      </c>
-      <c r="T8" s="216">
+        <v>4.2398280593728841E-7</v>
+      </c>
+      <c r="T8" s="221">
         <f t="shared" ref="T8" si="9">U8/SQRT(5)</f>
-        <v>4.4196755738981199E-7</v>
-      </c>
-      <c r="U8" s="228">
+        <v>4.2232455483915373E-7</v>
+      </c>
+      <c r="U8" s="227">
         <f t="shared" ref="U8" si="10">_xlfn.STDEV.S(O8:O12)</f>
-        <v>9.882695021731592E-7</v>
+        <v>9.4434641318768558E-7</v>
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
@@ -10319,14 +10465,14 @@
         <f t="shared" si="1"/>
         <v>294.09999999999997</v>
       </c>
-      <c r="G9" s="101">
+      <c r="G9" s="279">
         <v>25</v>
       </c>
-      <c r="H9" s="117">
+      <c r="H9" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I9" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I9" s="285">
         <v>0.28000000000000003</v>
       </c>
       <c r="J9" s="27">
@@ -10347,7 +10493,7 @@
       </c>
       <c r="O9" s="145">
         <f t="shared" si="4"/>
-        <v>2.5976708859512412E-6</v>
+        <v>2.482218846575631E-6</v>
       </c>
       <c r="P9" s="218"/>
       <c r="Q9" s="223"/>
@@ -10375,14 +10521,14 @@
         <f t="shared" si="1"/>
         <v>294.29999999999995</v>
       </c>
-      <c r="G10" s="101">
+      <c r="G10" s="279">
         <v>25</v>
       </c>
-      <c r="H10" s="117">
+      <c r="H10" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I10" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I10" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J10" s="27">
@@ -10403,7 +10549,7 @@
       </c>
       <c r="O10" s="145">
         <f t="shared" si="4"/>
-        <v>2.2553421645468143E-6</v>
+        <v>2.1551047350114005E-6</v>
       </c>
       <c r="P10" s="218"/>
       <c r="Q10" s="223"/>
@@ -10431,14 +10577,14 @@
         <f t="shared" si="1"/>
         <v>292.7</v>
       </c>
-      <c r="G11" s="101">
+      <c r="G11" s="279">
         <v>25</v>
       </c>
-      <c r="H11" s="117">
+      <c r="H11" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I11" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I11" s="285">
         <v>0.31</v>
       </c>
       <c r="J11" s="27">
@@ -10459,7 +10605,7 @@
       </c>
       <c r="O11" s="145">
         <f t="shared" si="4"/>
-        <v>2.4355635703895964E-6</v>
+        <v>2.3273163005945036E-6</v>
       </c>
       <c r="P11" s="218"/>
       <c r="Q11" s="223"/>
@@ -10469,60 +10615,60 @@
       <c r="U11" s="228"/>
     </row>
     <row r="12" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="207"/>
-      <c r="B12" s="133">
+      <c r="A12" s="208"/>
+      <c r="B12" s="132">
         <v>5</v>
       </c>
-      <c r="C12" s="161">
+      <c r="C12" s="140">
         <v>20</v>
       </c>
-      <c r="D12" s="162">
+      <c r="D12" s="54">
         <f t="shared" si="11"/>
         <v>293.14999999999998</v>
       </c>
-      <c r="E12" s="163">
+      <c r="E12" s="136">
         <v>19.55</v>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="183">
         <f t="shared" si="1"/>
         <v>292.7</v>
       </c>
-      <c r="G12" s="164">
+      <c r="G12" s="280">
         <v>25</v>
       </c>
-      <c r="H12" s="157">
+      <c r="H12" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I12" s="108">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I12" s="287">
         <v>0.31</v>
       </c>
-      <c r="J12" s="33">
+      <c r="J12" s="28">
         <v>32.799999999999997</v>
       </c>
-      <c r="K12" s="34">
+      <c r="K12" s="18">
         <v>60</v>
       </c>
-      <c r="L12" s="165">
+      <c r="L12" s="122">
         <v>0.57999999999999996</v>
       </c>
-      <c r="M12" s="34">
+      <c r="M12" s="18">
         <f t="shared" si="3"/>
         <v>21.323529411764703</v>
       </c>
-      <c r="N12" s="187">
+      <c r="N12" s="172">
         <v>0.46100000000000002</v>
       </c>
-      <c r="O12" s="166">
+      <c r="O12" s="147">
         <f t="shared" si="4"/>
-        <v>1.9694759658192417E-6</v>
-      </c>
-      <c r="P12" s="218"/>
+        <v>1.8819437006717198E-6</v>
+      </c>
+      <c r="P12" s="220"/>
       <c r="Q12" s="224"/>
       <c r="R12" s="224"/>
       <c r="S12" s="224"/>
-      <c r="T12" s="216"/>
-      <c r="U12" s="228"/>
+      <c r="T12" s="217"/>
+      <c r="U12" s="229"/>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A13" s="226">
@@ -10545,14 +10691,14 @@
         <f t="shared" si="1"/>
         <v>298.64999999999998</v>
       </c>
-      <c r="G13" s="112">
+      <c r="G13" s="276">
         <v>25</v>
       </c>
       <c r="H13" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I13" s="113">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I13" s="284">
         <v>0.28999999999999998</v>
       </c>
       <c r="J13" s="110">
@@ -10573,11 +10719,11 @@
       </c>
       <c r="O13" s="153">
         <f t="shared" si="4"/>
-        <v>3.8790863563648034E-6</v>
+        <v>3.7066825183041457E-6</v>
       </c>
       <c r="P13" s="219">
         <f t="shared" ref="P13" si="12">AVERAGE(O13:O17)</f>
-        <v>3.3903837799776504E-6</v>
+        <v>3.2397000564230882E-6</v>
       </c>
       <c r="Q13" s="222">
         <f t="shared" ref="Q13" si="13">AVERAGE(M13:M17)</f>
@@ -10589,15 +10735,15 @@
       </c>
       <c r="S13" s="222">
         <f t="shared" ref="S13" si="15">SQRT(T13^2+((SQRT((0.5/D13)^2+(R13/Q13)^2+(0.06/225)^2))*P13)^2)</f>
-        <v>2.8822893176888274E-7</v>
+        <v>2.7541875702359903E-7</v>
       </c>
       <c r="T13" s="221">
         <f t="shared" ref="T13" si="16">U13/SQRT(5)</f>
-        <v>2.8496029307747946E-7</v>
+        <v>2.7229539116292476E-7</v>
       </c>
       <c r="U13" s="227">
         <f t="shared" ref="U13" si="17">_xlfn.STDEV.S(O13:O17)</f>
-        <v>6.3719058620950689E-7</v>
+        <v>6.0887100460019533E-7</v>
       </c>
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.2">
@@ -10619,14 +10765,14 @@
         <f t="shared" si="1"/>
         <v>298.7</v>
       </c>
-      <c r="G14" s="101">
+      <c r="G14" s="279">
         <v>25</v>
       </c>
-      <c r="H14" s="117">
+      <c r="H14" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I14" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I14" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J14" s="27">
@@ -10647,7 +10793,7 @@
       </c>
       <c r="O14" s="145">
         <f t="shared" si="4"/>
-        <v>4.1871732874208404E-6</v>
+        <v>4.0010766968688024E-6</v>
       </c>
       <c r="P14" s="218"/>
       <c r="Q14" s="223"/>
@@ -10675,14 +10821,14 @@
         <f t="shared" si="1"/>
         <v>299.34999999999997</v>
       </c>
-      <c r="G15" s="101">
+      <c r="G15" s="279">
         <v>25</v>
       </c>
-      <c r="H15" s="117">
+      <c r="H15" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I15" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I15" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J15" s="27">
@@ -10703,7 +10849,7 @@
       </c>
       <c r="O15" s="145">
         <f t="shared" si="4"/>
-        <v>3.1678855587403213E-6</v>
+        <v>3.0270906450185293E-6</v>
       </c>
       <c r="P15" s="218"/>
       <c r="Q15" s="223"/>
@@ -10731,14 +10877,14 @@
         <f t="shared" si="1"/>
         <v>297.79999999999995</v>
       </c>
-      <c r="G16" s="101">
+      <c r="G16" s="279">
         <v>25</v>
       </c>
-      <c r="H16" s="117">
+      <c r="H16" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I16" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I16" s="285">
         <v>0.28000000000000003</v>
       </c>
       <c r="J16" s="27">
@@ -10759,7 +10905,7 @@
       </c>
       <c r="O16" s="145">
         <f t="shared" si="4"/>
-        <v>2.5982528036409038E-6</v>
+        <v>2.4827749012568637E-6</v>
       </c>
       <c r="P16" s="218"/>
       <c r="Q16" s="223"/>
@@ -10783,18 +10929,18 @@
       <c r="E17" s="136">
         <v>25.65</v>
       </c>
-      <c r="F17" s="29">
+      <c r="F17" s="183">
         <f t="shared" si="1"/>
         <v>298.79999999999995</v>
       </c>
-      <c r="G17" s="102">
+      <c r="G17" s="280">
         <v>25</v>
       </c>
-      <c r="H17" s="146">
+      <c r="H17" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I17" s="109">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I17" s="287">
         <v>0.3</v>
       </c>
       <c r="J17" s="28">
@@ -10815,7 +10961,7 @@
       </c>
       <c r="O17" s="147">
         <f t="shared" si="4"/>
-        <v>3.1195208937213843E-6</v>
+        <v>2.9808755206671005E-6</v>
       </c>
       <c r="P17" s="220"/>
       <c r="Q17" s="224"/>
@@ -10845,14 +10991,14 @@
         <f t="shared" si="1"/>
         <v>303.25</v>
       </c>
-      <c r="G18" s="112">
+      <c r="G18" s="276">
         <v>25</v>
       </c>
       <c r="H18" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I18" s="113">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I18" s="284">
         <v>0.33</v>
       </c>
       <c r="J18" s="110">
@@ -10873,11 +11019,11 @@
       </c>
       <c r="O18" s="153">
         <f t="shared" si="4"/>
-        <v>1.1021458798142964E-5</v>
+        <v>1.0531616184892166E-5</v>
       </c>
       <c r="P18" s="219">
         <f t="shared" ref="P18" si="18">AVERAGE(O18:O22)</f>
-        <v>7.5427965937800808E-6</v>
+        <v>7.2075611896120787E-6</v>
       </c>
       <c r="Q18" s="222">
         <f t="shared" ref="Q18" si="19">AVERAGE(M18:M22)</f>
@@ -10889,15 +11035,15 @@
       </c>
       <c r="S18" s="222">
         <f t="shared" ref="S18" si="21">SQRT(T18^2+((SQRT((0.5/D18)^2+(R18/Q18)^2+(0.06/225)^2))*P18)^2)</f>
-        <v>1.1955215397196222E-6</v>
+        <v>1.1423872490654169E-6</v>
       </c>
       <c r="T18" s="221">
         <f t="shared" ref="T18" si="22">U18/SQRT(5)</f>
-        <v>1.1928944000136995E-6</v>
+        <v>1.1398768711242019E-6</v>
       </c>
       <c r="U18" s="227">
         <f t="shared" ref="U18" si="23">_xlfn.STDEV.S(O18:O22)</f>
-        <v>2.6673929684094582E-6</v>
+        <v>2.5488421698134824E-6</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.2">
@@ -10919,14 +11065,14 @@
         <f t="shared" si="1"/>
         <v>301.95</v>
       </c>
-      <c r="G19" s="101">
+      <c r="G19" s="279">
         <v>25</v>
       </c>
-      <c r="H19" s="117">
+      <c r="H19" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I19" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I19" s="285">
         <v>0.3</v>
       </c>
       <c r="J19" s="27">
@@ -10947,7 +11093,7 @@
       </c>
       <c r="O19" s="145">
         <f t="shared" si="4"/>
-        <v>5.309061718904294E-6</v>
+        <v>5.0731034202863258E-6</v>
       </c>
       <c r="P19" s="218"/>
       <c r="Q19" s="223"/>
@@ -10975,14 +11121,14 @@
         <f t="shared" si="1"/>
         <v>304.34999999999997</v>
       </c>
-      <c r="G20" s="101">
+      <c r="G20" s="279">
         <v>25</v>
       </c>
-      <c r="H20" s="117">
+      <c r="H20" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I20" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I20" s="285">
         <v>0.3</v>
       </c>
       <c r="J20" s="27">
@@ -11003,7 +11149,7 @@
       </c>
       <c r="O20" s="145">
         <f t="shared" si="4"/>
-        <v>9.7295510154863137E-6</v>
+        <v>9.2971265259091457E-6</v>
       </c>
       <c r="P20" s="218"/>
       <c r="Q20" s="223"/>
@@ -11031,14 +11177,14 @@
         <f t="shared" si="1"/>
         <v>303.34999999999997</v>
       </c>
-      <c r="G21" s="101">
+      <c r="G21" s="279">
         <v>25</v>
       </c>
-      <c r="H21" s="117">
+      <c r="H21" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I21" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I21" s="285">
         <v>0.3</v>
       </c>
       <c r="J21" s="27">
@@ -11059,7 +11205,7 @@
       </c>
       <c r="O21" s="145">
         <f t="shared" si="4"/>
-        <v>6.4182103362598011E-6</v>
+        <v>6.1329565435371442E-6</v>
       </c>
       <c r="P21" s="218"/>
       <c r="Q21" s="223"/>
@@ -11083,18 +11229,18 @@
       <c r="E22" s="136">
         <v>30.9</v>
       </c>
-      <c r="F22" s="29">
+      <c r="F22" s="183">
         <f t="shared" si="1"/>
         <v>304.04999999999995</v>
       </c>
-      <c r="G22" s="102">
+      <c r="G22" s="280">
         <v>25</v>
       </c>
-      <c r="H22" s="146">
+      <c r="H22" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I22" s="109">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I22" s="287">
         <v>0.28999999999999998</v>
       </c>
       <c r="J22" s="28">
@@ -11115,7 +11261,7 @@
       </c>
       <c r="O22" s="147">
         <f t="shared" si="4"/>
-        <v>5.2357011001070352E-6</v>
+        <v>5.0030032734356118E-6</v>
       </c>
       <c r="P22" s="220"/>
       <c r="Q22" s="224"/>
@@ -11125,59 +11271,59 @@
       <c r="U22" s="229"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A23" s="198">
+      <c r="A23" s="226">
         <v>5</v>
       </c>
-      <c r="B23" s="148">
+      <c r="B23" s="129">
         <v>1</v>
       </c>
-      <c r="C23" s="149">
+      <c r="C23" s="138">
         <v>35</v>
       </c>
-      <c r="D23" s="159">
+      <c r="D23" s="52">
         <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
-      <c r="E23" s="135">
+      <c r="E23" s="134">
         <v>35.5</v>
       </c>
       <c r="F23" s="182">
         <f t="shared" si="1"/>
         <v>308.64999999999998</v>
       </c>
-      <c r="G23" s="100">
+      <c r="G23" s="276">
         <v>25</v>
       </c>
-      <c r="H23" s="117">
+      <c r="H23" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I23" s="119">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I23" s="284">
         <v>0.31</v>
       </c>
-      <c r="J23" s="25">
+      <c r="J23" s="110">
         <v>7.8</v>
       </c>
-      <c r="K23" s="19">
+      <c r="K23" s="111">
         <v>60</v>
       </c>
-      <c r="L23" s="150">
+      <c r="L23" s="120">
         <v>6.12</v>
       </c>
-      <c r="M23" s="19">
+      <c r="M23" s="111">
         <f t="shared" si="3"/>
         <v>117.24137931034483</v>
       </c>
-      <c r="N23" s="186">
+      <c r="N23" s="170">
         <v>0.90200000000000002</v>
       </c>
-      <c r="O23" s="151">
+      <c r="O23" s="153">
         <f t="shared" si="4"/>
-        <v>1.0301494651938654E-5</v>
-      </c>
-      <c r="P23" s="218">
+        <v>9.8436504451858246E-6</v>
+      </c>
+      <c r="P23" s="219">
         <f t="shared" ref="P23" si="24">AVERAGE(O23:O27)</f>
-        <v>8.5940925905051713E-6</v>
+        <v>8.2121329198160521E-6</v>
       </c>
       <c r="Q23" s="222">
         <f t="shared" ref="Q23" si="25">AVERAGE(M23:M27)</f>
@@ -11189,15 +11335,15 @@
       </c>
       <c r="S23" s="222">
         <f t="shared" ref="S23" si="27">SQRT(T23^2+((SQRT((0.5/D23)^2+(R23/Q23)^2+(0.06/225)^2))*P23)^2)</f>
-        <v>9.2923209561911543E-7</v>
-      </c>
-      <c r="T23" s="216">
+        <v>8.8793289136937687E-7</v>
+      </c>
+      <c r="T23" s="221">
         <f t="shared" ref="T23" si="28">U23/SQRT(5)</f>
-        <v>9.2616602094664455E-7</v>
-      </c>
-      <c r="U23" s="228">
+        <v>8.8500308668234917E-7</v>
+      </c>
+      <c r="U23" s="227">
         <f t="shared" ref="U23" si="29">_xlfn.STDEV.S(O23:O27)</f>
-        <v>2.0709701812871915E-6</v>
+        <v>1.9789270621188717E-6</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.2">
@@ -11219,14 +11365,14 @@
         <f t="shared" si="1"/>
         <v>308.7</v>
       </c>
-      <c r="G24" s="101">
+      <c r="G24" s="279">
         <v>25</v>
       </c>
-      <c r="H24" s="117">
+      <c r="H24" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I24" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I24" s="285">
         <v>0.31</v>
       </c>
       <c r="J24" s="27">
@@ -11247,7 +11393,7 @@
       </c>
       <c r="O24" s="145">
         <f t="shared" si="4"/>
-        <v>7.8509620869962748E-6</v>
+        <v>7.5020304386853293E-6</v>
       </c>
       <c r="P24" s="218"/>
       <c r="Q24" s="223"/>
@@ -11275,14 +11421,14 @@
         <f t="shared" si="1"/>
         <v>307.34999999999997</v>
       </c>
-      <c r="G25" s="101">
+      <c r="G25" s="279">
         <v>25</v>
       </c>
-      <c r="H25" s="117">
+      <c r="H25" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I25" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I25" s="285">
         <v>0.32</v>
       </c>
       <c r="J25" s="27">
@@ -11303,7 +11449,7 @@
       </c>
       <c r="O25" s="145">
         <f t="shared" si="4"/>
-        <v>8.8653722769585487E-6</v>
+        <v>8.4713557313159462E-6</v>
       </c>
       <c r="P25" s="218"/>
       <c r="Q25" s="223"/>
@@ -11331,14 +11477,14 @@
         <f t="shared" si="1"/>
         <v>308.14999999999998</v>
       </c>
-      <c r="G26" s="101">
+      <c r="G26" s="279">
         <v>25</v>
       </c>
-      <c r="H26" s="117">
+      <c r="H26" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I26" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I26" s="285">
         <v>0.31</v>
       </c>
       <c r="J26" s="27">
@@ -11359,7 +11505,7 @@
       </c>
       <c r="O26" s="145">
         <f t="shared" si="4"/>
-        <v>1.0511205438788404E-5</v>
+        <v>1.0044040752620029E-5</v>
       </c>
       <c r="P26" s="218"/>
       <c r="Q26" s="223"/>
@@ -11369,60 +11515,60 @@
       <c r="U26" s="228"/>
     </row>
     <row r="27" spans="1:21" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="207"/>
-      <c r="B27" s="133">
+      <c r="A27" s="208"/>
+      <c r="B27" s="132">
         <v>5</v>
       </c>
-      <c r="C27" s="161">
+      <c r="C27" s="140">
         <v>35</v>
       </c>
-      <c r="D27" s="162">
+      <c r="D27" s="54">
         <f t="shared" si="11"/>
         <v>308.14999999999998</v>
       </c>
-      <c r="E27" s="163">
+      <c r="E27" s="136">
         <v>35.9</v>
       </c>
-      <c r="F27" s="29">
+      <c r="F27" s="183">
         <f t="shared" si="1"/>
         <v>309.04999999999995</v>
       </c>
-      <c r="G27" s="164">
+      <c r="G27" s="280">
         <v>25</v>
       </c>
-      <c r="H27" s="157">
+      <c r="H27" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I27" s="108">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I27" s="287">
         <v>0.28999999999999998</v>
       </c>
-      <c r="J27" s="33">
+      <c r="J27" s="28">
         <v>20.6</v>
       </c>
-      <c r="K27" s="34">
+      <c r="K27" s="18">
         <v>60</v>
       </c>
-      <c r="L27" s="165">
+      <c r="L27" s="122">
         <v>2.44</v>
       </c>
-      <c r="M27" s="34">
+      <c r="M27" s="18">
         <f t="shared" si="3"/>
         <v>61.92893401015229</v>
       </c>
-      <c r="N27" s="187">
+      <c r="N27" s="172">
         <v>0.67800000000000005</v>
       </c>
-      <c r="O27" s="166">
+      <c r="O27" s="147">
         <f t="shared" si="4"/>
-        <v>5.4414284978439773E-6</v>
-      </c>
-      <c r="P27" s="218"/>
+        <v>5.1995872312731344E-6</v>
+      </c>
+      <c r="P27" s="220"/>
       <c r="Q27" s="224"/>
       <c r="R27" s="224"/>
       <c r="S27" s="224"/>
-      <c r="T27" s="216"/>
-      <c r="U27" s="228"/>
+      <c r="T27" s="217"/>
+      <c r="U27" s="229"/>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" s="226">
@@ -11445,14 +11591,14 @@
         <f t="shared" si="1"/>
         <v>313.5</v>
       </c>
-      <c r="G28" s="112">
+      <c r="G28" s="276">
         <v>25</v>
       </c>
       <c r="H28" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I28" s="113">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I28" s="284">
         <v>0.28000000000000003</v>
       </c>
       <c r="J28" s="110">
@@ -11473,11 +11619,11 @@
       </c>
       <c r="O28" s="153">
         <f t="shared" si="4"/>
-        <v>9.8156490238009875E-6</v>
+        <v>9.3793979560764982E-6</v>
       </c>
       <c r="P28" s="219">
         <f t="shared" ref="P28" si="30">AVERAGE(O28:O32)</f>
-        <v>8.8862471284774915E-6</v>
+        <v>8.4913028116562706E-6</v>
       </c>
       <c r="Q28" s="222">
         <f t="shared" ref="Q28" si="31">AVERAGE(M28:M32)</f>
@@ -11489,15 +11635,15 @@
       </c>
       <c r="S28" s="222">
         <f t="shared" ref="S28" si="33">SQRT(T28^2+((SQRT((0.5/D28)^2+(R28/Q28)^2+(0.06/225)^2))*P28)^2)</f>
-        <v>1.2117876573322692E-6</v>
+        <v>1.1579304281175019E-6</v>
       </c>
       <c r="T28" s="221">
         <f t="shared" ref="T28" si="34">U28/SQRT(5)</f>
-        <v>1.2081347586731623E-6</v>
+        <v>1.1544398805099108E-6</v>
       </c>
       <c r="U28" s="227">
         <f t="shared" ref="U28" si="35">_xlfn.STDEV.S(O28:O32)</f>
-        <v>2.7014714463734948E-6</v>
+        <v>2.5814060487568954E-6</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.2">
@@ -11519,14 +11665,14 @@
         <f t="shared" si="1"/>
         <v>314.34999999999997</v>
       </c>
-      <c r="G29" s="101">
+      <c r="G29" s="279">
         <v>25</v>
       </c>
-      <c r="H29" s="117">
+      <c r="H29" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I29" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I29" s="285">
         <v>0.28000000000000003</v>
       </c>
       <c r="J29" s="27">
@@ -11547,7 +11693,7 @@
       </c>
       <c r="O29" s="145">
         <f t="shared" si="4"/>
-        <v>8.1868117496687828E-6</v>
+        <v>7.8229534496835042E-6</v>
       </c>
       <c r="P29" s="218"/>
       <c r="Q29" s="223"/>
@@ -11575,14 +11721,14 @@
         <f t="shared" si="1"/>
         <v>312.04999999999995</v>
       </c>
-      <c r="G30" s="101">
+      <c r="G30" s="279">
         <v>25</v>
       </c>
-      <c r="H30" s="117">
+      <c r="H30" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I30" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I30" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J30" s="27">
@@ -11603,7 +11749,7 @@
       </c>
       <c r="O30" s="145">
         <f t="shared" si="4"/>
-        <v>6.2379523130339029E-6</v>
+        <v>5.9607099880101735E-6</v>
       </c>
       <c r="P30" s="218"/>
       <c r="Q30" s="223"/>
@@ -11631,14 +11777,14 @@
         <f t="shared" si="1"/>
         <v>313.64999999999998</v>
       </c>
-      <c r="G31" s="101">
+      <c r="G31" s="279">
         <v>25</v>
       </c>
-      <c r="H31" s="117">
+      <c r="H31" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I31" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I31" s="285">
         <v>0.28000000000000003</v>
       </c>
       <c r="J31" s="27">
@@ -11659,7 +11805,7 @@
       </c>
       <c r="O31" s="145">
         <f t="shared" si="4"/>
-        <v>1.3087164347625258E-5</v>
+        <v>1.2505512598841914E-5</v>
       </c>
       <c r="P31" s="218"/>
       <c r="Q31" s="223"/>
@@ -11683,18 +11829,18 @@
       <c r="E32" s="136">
         <v>38.950000000000003</v>
       </c>
-      <c r="F32" s="29">
+      <c r="F32" s="183">
         <f t="shared" si="1"/>
         <v>312.09999999999997</v>
       </c>
-      <c r="G32" s="102">
+      <c r="G32" s="280">
         <v>25</v>
       </c>
-      <c r="H32" s="146">
+      <c r="H32" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I32" s="109">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I32" s="287">
         <v>0.28999999999999998</v>
       </c>
       <c r="J32" s="28">
@@ -11715,7 +11861,7 @@
       </c>
       <c r="O32" s="147">
         <f t="shared" si="4"/>
-        <v>7.1036582082585224E-6</v>
+        <v>6.7879400656692549E-6</v>
       </c>
       <c r="P32" s="220"/>
       <c r="Q32" s="224"/>
@@ -11745,14 +11891,14 @@
         <f t="shared" si="1"/>
         <v>318.39999999999998</v>
       </c>
-      <c r="G33" s="112">
+      <c r="G33" s="276">
         <v>25</v>
       </c>
       <c r="H33" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I33" s="113">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I33" s="284">
         <v>0.28999999999999998</v>
       </c>
       <c r="J33" s="110">
@@ -11773,11 +11919,11 @@
       </c>
       <c r="O33" s="153">
         <f t="shared" si="4"/>
-        <v>1.1352541834116659E-5</v>
+        <v>1.0847984419267031E-5</v>
       </c>
       <c r="P33" s="219">
         <f t="shared" ref="P33" si="36">AVERAGE(O33:O37)</f>
-        <v>1.2906068842991905E-5</v>
+        <v>1.2332465783303374E-5</v>
       </c>
       <c r="Q33" s="222">
         <f t="shared" ref="Q33" si="37">AVERAGE(M33:M37)</f>
@@ -11789,15 +11935,15 @@
       </c>
       <c r="S33" s="222">
         <f t="shared" ref="S33" si="39">SQRT(T33^2+((SQRT((0.5/D33)^2+(R33/Q33)^2+(0.06/225)^2))*P33)^2)</f>
-        <v>2.711288692750651E-6</v>
+        <v>2.5907869730728439E-6</v>
       </c>
       <c r="T33" s="221">
         <f t="shared" ref="T33" si="40">U33/SQRT(5)</f>
-        <v>2.7092205631905007E-6</v>
+        <v>2.5888107603820336E-6</v>
       </c>
       <c r="U33" s="227">
         <f t="shared" ref="U33" si="41">_xlfn.STDEV.S(O33:O37)</f>
-        <v>6.0580013453342243E-6</v>
+        <v>5.788756841097147E-6</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.2">
@@ -11819,14 +11965,14 @@
         <f t="shared" si="1"/>
         <v>317</v>
       </c>
-      <c r="G34" s="101">
+      <c r="G34" s="279">
         <v>25</v>
       </c>
-      <c r="H34" s="117">
+      <c r="H34" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I34" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I34" s="285">
         <v>0.3</v>
       </c>
       <c r="J34" s="27">
@@ -11847,7 +11993,7 @@
       </c>
       <c r="O34" s="145">
         <f t="shared" si="4"/>
-        <v>9.4082774384057253E-6</v>
+        <v>8.9901317744765814E-6</v>
       </c>
       <c r="P34" s="218"/>
       <c r="Q34" s="223"/>
@@ -11875,14 +12021,14 @@
         <f t="shared" si="1"/>
         <v>317.95</v>
       </c>
-      <c r="G35" s="101">
+      <c r="G35" s="279">
         <v>25</v>
       </c>
-      <c r="H35" s="117">
+      <c r="H35" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I35" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I35" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J35" s="27">
@@ -11903,7 +12049,7 @@
       </c>
       <c r="O35" s="145">
         <f t="shared" si="4"/>
-        <v>1.7788870003601831E-5</v>
+        <v>1.6998253558997307E-5</v>
       </c>
       <c r="P35" s="218"/>
       <c r="Q35" s="223"/>
@@ -11931,14 +12077,14 @@
         <f t="shared" si="1"/>
         <v>317.75</v>
       </c>
-      <c r="G36" s="101">
+      <c r="G36" s="279">
         <v>25</v>
       </c>
-      <c r="H36" s="117">
+      <c r="H36" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I36" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I36" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J36" s="27">
@@ -11959,7 +12105,7 @@
       </c>
       <c r="O36" s="145">
         <f t="shared" si="4"/>
-        <v>2.0348777853726677E-5</v>
+        <v>1.9444387726894379E-5</v>
       </c>
       <c r="P36" s="218"/>
       <c r="Q36" s="223"/>
@@ -11983,18 +12129,18 @@
       <c r="E37" s="136">
         <v>44.650000000000006</v>
       </c>
-      <c r="F37" s="29">
+      <c r="F37" s="183">
         <f t="shared" si="1"/>
         <v>317.79999999999995</v>
       </c>
-      <c r="G37" s="102">
+      <c r="G37" s="280">
         <v>25</v>
       </c>
-      <c r="H37" s="146">
+      <c r="H37" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I37" s="109">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I37" s="287">
         <v>0.28999999999999998</v>
       </c>
       <c r="J37" s="28">
@@ -12015,7 +12161,7 @@
       </c>
       <c r="O37" s="147">
         <f t="shared" si="4"/>
-        <v>5.6318770851086252E-6</v>
+        <v>5.3815714368815754E-6</v>
       </c>
       <c r="P37" s="220"/>
       <c r="Q37" s="224"/>
@@ -12025,59 +12171,59 @@
       <c r="U37" s="229"/>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A38" s="198">
+      <c r="A38" s="226">
         <v>8</v>
       </c>
-      <c r="B38" s="148">
+      <c r="B38" s="129">
         <v>1</v>
       </c>
-      <c r="C38" s="149">
+      <c r="C38" s="138">
         <v>50</v>
       </c>
-      <c r="D38" s="159">
+      <c r="D38" s="52">
         <f t="shared" si="11"/>
         <v>323.14999999999998</v>
       </c>
-      <c r="E38" s="135">
+      <c r="E38" s="134">
         <v>49.3</v>
       </c>
       <c r="F38" s="182">
         <f t="shared" si="1"/>
         <v>322.45</v>
       </c>
-      <c r="G38" s="100">
+      <c r="G38" s="276">
         <v>25</v>
       </c>
-      <c r="H38" s="117">
+      <c r="H38" s="152">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I38" s="119">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I38" s="284">
         <v>0.31</v>
       </c>
-      <c r="J38" s="25">
+      <c r="J38" s="110">
         <v>10.4</v>
       </c>
-      <c r="K38" s="19">
+      <c r="K38" s="111">
         <v>60</v>
       </c>
-      <c r="L38" s="150">
+      <c r="L38" s="120">
         <v>18.27</v>
       </c>
-      <c r="M38" s="19">
+      <c r="M38" s="111">
         <f t="shared" si="3"/>
         <v>368.34677419354841</v>
       </c>
-      <c r="N38" s="186">
+      <c r="N38" s="170">
         <v>1.637</v>
       </c>
-      <c r="O38" s="151">
+      <c r="O38" s="153">
         <f t="shared" si="4"/>
-        <v>3.0862720439219007E-5</v>
-      </c>
-      <c r="P38" s="218">
+        <v>2.9491043975253719E-5</v>
+      </c>
+      <c r="P38" s="219">
         <f t="shared" ref="P38" si="42">AVERAGE(O38:O42)</f>
-        <v>1.843359308412242E-5</v>
+        <v>1.7614322280383645E-5</v>
       </c>
       <c r="Q38" s="222">
         <f t="shared" ref="Q38" si="43">AVERAGE(M38:M42)</f>
@@ -12089,15 +12235,15 @@
       </c>
       <c r="S38" s="222">
         <f t="shared" ref="S38" si="45">SQRT(T38^2+((SQRT((0.5/D38)^2+(R38/Q38)^2+(0.06/225)^2))*P38)^2)</f>
-        <v>3.820488923827413E-6</v>
-      </c>
-      <c r="T38" s="216">
+        <v>3.6506894161017504E-6</v>
+      </c>
+      <c r="T38" s="221">
         <f t="shared" ref="T38" si="46">U38/SQRT(5)</f>
-        <v>3.8173859957856402E-6</v>
-      </c>
-      <c r="U38" s="228">
+        <v>3.6477243959729456E-6</v>
+      </c>
+      <c r="U38" s="227">
         <f t="shared" ref="U38" si="47">_xlfn.STDEV.S(O38:O42)</f>
-        <v>8.5359345829324183E-6</v>
+        <v>8.1565597125798673E-6</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.2">
@@ -12119,14 +12265,14 @@
         <f t="shared" si="1"/>
         <v>322.54999999999995</v>
       </c>
-      <c r="G39" s="101">
+      <c r="G39" s="279">
         <v>25</v>
       </c>
-      <c r="H39" s="117">
+      <c r="H39" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I39" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I39" s="285">
         <v>0.28000000000000003</v>
       </c>
       <c r="J39" s="27">
@@ -12147,7 +12293,7 @@
       </c>
       <c r="O39" s="145">
         <f t="shared" si="4"/>
-        <v>1.1629376034248156E-5</v>
+        <v>1.111251487717046E-5</v>
       </c>
       <c r="P39" s="218"/>
       <c r="Q39" s="223"/>
@@ -12175,14 +12321,14 @@
         <f t="shared" si="1"/>
         <v>321.7</v>
       </c>
-      <c r="G40" s="101">
+      <c r="G40" s="279">
         <v>25</v>
       </c>
-      <c r="H40" s="117">
+      <c r="H40" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I40" s="107">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I40" s="285">
         <v>0.28999999999999998</v>
       </c>
       <c r="J40" s="27">
@@ -12203,7 +12349,7 @@
       </c>
       <c r="O40" s="145">
         <f t="shared" si="4"/>
-        <v>1.1948773857870259E-5</v>
+        <v>1.1417717241964913E-5</v>
       </c>
       <c r="P40" s="218"/>
       <c r="Q40" s="223"/>
@@ -12231,14 +12377,14 @@
         <f t="shared" si="1"/>
         <v>322.59999999999997</v>
       </c>
-      <c r="G41" s="101">
+      <c r="G41" s="279">
         <v>25</v>
       </c>
-      <c r="H41" s="117">
+      <c r="H41" s="281">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I41" s="108">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I41" s="288">
         <v>0.28999999999999998</v>
       </c>
       <c r="J41" s="27">
@@ -12259,7 +12405,7 @@
       </c>
       <c r="O41" s="145">
         <f t="shared" si="4"/>
-        <v>2.3775041119508106E-5</v>
+        <v>2.2718372625307744E-5</v>
       </c>
       <c r="P41" s="218"/>
       <c r="Q41" s="223"/>
@@ -12287,14 +12433,14 @@
         <f t="shared" si="1"/>
         <v>322.95</v>
       </c>
-      <c r="G42" s="102">
+      <c r="G42" s="280">
         <v>25</v>
       </c>
-      <c r="H42" s="146">
+      <c r="H42" s="282">
         <f t="shared" si="2"/>
-        <v>2.2499999999999999E-4</v>
-      </c>
-      <c r="I42" s="109">
+        <v>2.1499999999999999E-4</v>
+      </c>
+      <c r="I42" s="287">
         <v>0.28999999999999998</v>
       </c>
       <c r="J42" s="28">
@@ -12315,7 +12461,7 @@
       </c>
       <c r="O42" s="147">
         <f t="shared" si="4"/>
-        <v>1.3952053969766572E-5</v>
+        <v>1.3331962682221389E-5</v>
       </c>
       <c r="P42" s="220"/>
       <c r="Q42" s="224"/>
@@ -12396,7 +12542,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50153C52-BBF2-284B-968B-83E46E40C2E9}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:AV44"/>
+  <dimension ref="A1:BG44"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.5" style="1" customWidth="1"/>
@@ -12429,10 +12575,12 @@
     <col min="38" max="39" width="10.83203125" style="1"/>
     <col min="40" max="40" width="7.1640625" style="1" customWidth="1"/>
     <col min="41" max="41" width="21.6640625" style="1" customWidth="1"/>
-    <col min="42" max="16384" width="10.83203125" style="1"/>
+    <col min="42" max="56" width="10.83203125" style="1"/>
+    <col min="57" max="57" width="24.6640625" style="1" customWidth="1"/>
+    <col min="58" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" ht="20" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:56" ht="20" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="254" t="s">
         <v>14</v>
       </c>
@@ -12486,7 +12634,7 @@
       <c r="AU1" s="190"/>
       <c r="AV1" s="190"/>
     </row>
-    <row r="2" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:56" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -12598,7 +12746,7 @@
       <c r="AU2" s="137"/>
       <c r="AV2" s="192"/>
     </row>
-    <row r="3" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="226">
         <v>1</v>
       </c>
@@ -12728,7 +12876,7 @@
       <c r="AU3" s="193"/>
       <c r="AV3" s="194"/>
     </row>
-    <row r="4" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="195"/>
       <c r="B4" s="130">
         <v>2</v>
@@ -12815,7 +12963,7 @@
       <c r="AU4" s="193"/>
       <c r="AV4" s="194"/>
     </row>
-    <row r="5" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="195"/>
       <c r="B5" s="130">
         <v>3</v>
@@ -12902,7 +13050,7 @@
       <c r="AU5" s="193"/>
       <c r="AV5" s="194"/>
     </row>
-    <row r="6" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="195"/>
       <c r="B6" s="130">
         <v>4</v>
@@ -12989,7 +13137,7 @@
       <c r="AU6" s="193"/>
       <c r="AV6" s="194"/>
     </row>
-    <row r="7" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:56" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="208"/>
       <c r="B7" s="131">
         <v>5</v>
@@ -12997,14 +13145,14 @@
       <c r="C7" s="154">
         <v>15</v>
       </c>
-      <c r="D7" s="54">
+      <c r="D7" s="63">
         <f t="shared" si="0"/>
         <v>288.14999999999998</v>
       </c>
       <c r="E7" s="141">
         <v>14.86</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="275">
         <f t="shared" si="1"/>
         <v>288.01</v>
       </c>
@@ -13076,7 +13224,7 @@
       <c r="AU7" s="193"/>
       <c r="AV7" s="194"/>
     </row>
-    <row r="8" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="198">
         <v>2</v>
       </c>
@@ -13206,7 +13354,7 @@
       <c r="AU8" s="193"/>
       <c r="AV8" s="194"/>
     </row>
-    <row r="9" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="195"/>
       <c r="B9" s="130">
         <v>2</v>
@@ -13293,7 +13441,7 @@
       <c r="AU9" s="193"/>
       <c r="AV9" s="194"/>
     </row>
-    <row r="10" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="195"/>
       <c r="B10" s="130">
         <v>3</v>
@@ -13380,7 +13528,7 @@
       <c r="AU10" s="193"/>
       <c r="AV10" s="194"/>
     </row>
-    <row r="11" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="195"/>
       <c r="B11" s="130">
         <v>4</v>
@@ -13466,8 +13614,14 @@
       <c r="AT11" s="231"/>
       <c r="AU11" s="193"/>
       <c r="AV11" s="194"/>
+      <c r="BC11" s="99" t="s">
+        <v>70</v>
+      </c>
+      <c r="BD11" s="99" t="s">
+        <v>71</v>
+      </c>
     </row>
-    <row r="12" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:56" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="207"/>
       <c r="B12" s="133">
         <v>5</v>
@@ -13553,8 +13707,14 @@
       <c r="AT12" s="232"/>
       <c r="AU12" s="193"/>
       <c r="AV12" s="194"/>
+      <c r="BC12" s="1">
+        <v>3.4704147145583901E-3</v>
+      </c>
+      <c r="BD12" s="1">
+        <v>-13.180753833192105</v>
+      </c>
     </row>
-    <row r="13" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="226">
         <v>3</v>
       </c>
@@ -13683,8 +13843,14 @@
       </c>
       <c r="AU13" s="193"/>
       <c r="AV13" s="194"/>
+      <c r="BC13" s="1">
+        <v>3.4112229234180458E-3</v>
+      </c>
+      <c r="BD13" s="1">
+        <v>-13.181573232616515</v>
+      </c>
     </row>
-    <row r="14" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="195"/>
       <c r="B14" s="130">
         <v>2</v>
@@ -13770,8 +13936,14 @@
       <c r="AT14" s="231"/>
       <c r="AU14" s="193"/>
       <c r="AV14" s="194"/>
+      <c r="BC14" s="1">
+        <v>3.3540164346805303E-3</v>
+      </c>
+      <c r="BD14" s="1">
+        <v>-12.594567433546684</v>
+      </c>
     </row>
-    <row r="15" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="195"/>
       <c r="B15" s="130">
         <v>3</v>
@@ -13857,8 +14029,14 @@
       <c r="AT15" s="231"/>
       <c r="AU15" s="193"/>
       <c r="AV15" s="194"/>
+      <c r="BC15" s="1">
+        <v>3.298697014679202E-3</v>
+      </c>
+      <c r="BD15" s="1">
+        <v>-11.794917543679352</v>
+      </c>
     </row>
-    <row r="16" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:56" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="195"/>
       <c r="B16" s="130">
         <v>4</v>
@@ -13944,8 +14122,14 @@
       <c r="AT16" s="231"/>
       <c r="AU16" s="193"/>
       <c r="AV16" s="194"/>
+      <c r="BC16" s="1">
+        <v>3.2451728054518907E-3</v>
+      </c>
+      <c r="BD16" s="1">
+        <v>-11.664435498815054</v>
+      </c>
     </row>
-    <row r="17" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A17" s="208"/>
       <c r="B17" s="132">
         <v>5</v>
@@ -14031,8 +14215,14 @@
       <c r="AT17" s="232"/>
       <c r="AU17" s="193"/>
       <c r="AV17" s="194"/>
+      <c r="BC17" s="1">
+        <v>3.1933578157432542E-3</v>
+      </c>
+      <c r="BD17" s="1">
+        <v>-11.631005742844986</v>
+      </c>
     </row>
-    <row r="18" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="226">
         <v>4</v>
       </c>
@@ -14161,8 +14351,14 @@
       </c>
       <c r="AU18" s="193"/>
       <c r="AV18" s="194"/>
+      <c r="BC18" s="1">
+        <v>3.1431714600031434E-3</v>
+      </c>
+      <c r="BD18" s="1">
+        <v>-11.257812904279829</v>
+      </c>
     </row>
-    <row r="19" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="195"/>
       <c r="B19" s="130">
         <v>2</v>
@@ -14248,8 +14444,14 @@
       <c r="AT19" s="231"/>
       <c r="AU19" s="193"/>
       <c r="AV19" s="194"/>
+      <c r="BC19" s="1">
+        <v>3.0945381401825778E-3</v>
+      </c>
+      <c r="BD19" s="1">
+        <v>-10.901335846840498</v>
+      </c>
     </row>
-    <row r="20" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="195"/>
       <c r="B20" s="130">
         <v>3</v>
@@ -14336,7 +14538,7 @@
       <c r="AU20" s="193"/>
       <c r="AV20" s="194"/>
     </row>
-    <row r="21" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="195"/>
       <c r="B21" s="130">
         <v>4</v>
@@ -14423,7 +14625,7 @@
       <c r="AU21" s="193"/>
       <c r="AV21" s="194"/>
     </row>
-    <row r="22" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A22" s="208"/>
       <c r="B22" s="132">
         <v>5</v>
@@ -14510,7 +14712,7 @@
       <c r="AU22" s="193"/>
       <c r="AV22" s="194"/>
     </row>
-    <row r="23" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="198">
         <v>5</v>
       </c>
@@ -14640,7 +14842,7 @@
       <c r="AU23" s="193"/>
       <c r="AV23" s="194"/>
     </row>
-    <row r="24" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="195"/>
       <c r="B24" s="130">
         <v>2</v>
@@ -14727,7 +14929,7 @@
       <c r="AU24" s="193"/>
       <c r="AV24" s="194"/>
     </row>
-    <row r="25" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="195"/>
       <c r="B25" s="130">
         <v>3</v>
@@ -14814,7 +15016,7 @@
       <c r="AU25" s="193"/>
       <c r="AV25" s="194"/>
     </row>
-    <row r="26" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="195"/>
       <c r="B26" s="130">
         <v>4</v>
@@ -14901,7 +15103,7 @@
       <c r="AU26" s="193"/>
       <c r="AV26" s="194"/>
     </row>
-    <row r="27" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A27" s="207"/>
       <c r="B27" s="133">
         <v>5</v>
@@ -14988,7 +15190,7 @@
       <c r="AU27" s="193"/>
       <c r="AV27" s="194"/>
     </row>
-    <row r="28" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="226">
         <v>6</v>
       </c>
@@ -15118,7 +15320,7 @@
       <c r="AU28" s="193"/>
       <c r="AV28" s="194"/>
     </row>
-    <row r="29" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="195"/>
       <c r="B29" s="130">
         <v>2</v>
@@ -15205,7 +15407,7 @@
       <c r="AU29" s="193"/>
       <c r="AV29" s="194"/>
     </row>
-    <row r="30" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="195"/>
       <c r="B30" s="130">
         <v>3</v>
@@ -15292,7 +15494,7 @@
       <c r="AU30" s="193"/>
       <c r="AV30" s="194"/>
     </row>
-    <row r="31" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:57" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="195"/>
       <c r="B31" s="130">
         <v>4</v>
@@ -15379,7 +15581,7 @@
       <c r="AU31" s="193"/>
       <c r="AV31" s="194"/>
     </row>
-    <row r="32" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:57" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="208"/>
       <c r="B32" s="132">
         <v>5</v>
@@ -15465,8 +15667,9 @@
       <c r="AT32" s="232"/>
       <c r="AU32" s="193"/>
       <c r="AV32" s="194"/>
+      <c r="BE32" s="99"/>
     </row>
-    <row r="33" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="226">
         <v>7</v>
       </c>
@@ -15595,8 +15798,18 @@
       </c>
       <c r="AU33" s="193"/>
       <c r="AV33" s="194"/>
+      <c r="BE33" s="99" t="s">
+        <v>72</v>
+      </c>
+      <c r="BF33" s="1" cm="1">
+        <f t="array" ref="BF33:BG37">LINEST(BD12:BD19,BC12:BC19,TRUE,TRUE)</f>
+        <v>-6360.0109549020781</v>
+      </c>
+      <c r="BG33" s="1">
+        <v>8.8116557277608134</v>
+      </c>
     </row>
-    <row r="34" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="195"/>
       <c r="B34" s="130">
         <v>2</v>
@@ -15682,8 +15895,17 @@
       <c r="AT34" s="231"/>
       <c r="AU34" s="193"/>
       <c r="AV34" s="194"/>
+      <c r="BE34" s="99" t="s">
+        <v>73</v>
+      </c>
+      <c r="BF34" s="1">
+        <v>633.41550002975225</v>
+      </c>
+      <c r="BG34" s="1">
+        <v>2.0767363257166869</v>
+      </c>
     </row>
-    <row r="35" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="195"/>
       <c r="B35" s="130">
         <v>3</v>
@@ -15769,8 +15991,15 @@
       <c r="AT35" s="231"/>
       <c r="AU35" s="193"/>
       <c r="AV35" s="194"/>
+      <c r="BE35" s="99"/>
+      <c r="BF35" s="1">
+        <v>0.94382972537227494</v>
+      </c>
+      <c r="BG35" s="1">
+        <v>0.22036585656073118</v>
+      </c>
     </row>
-    <row r="36" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="195"/>
       <c r="B36" s="130">
         <v>4</v>
@@ -15856,8 +16085,14 @@
       <c r="AT36" s="231"/>
       <c r="AU36" s="193"/>
       <c r="AV36" s="194"/>
+      <c r="BF36" s="1">
+        <v>100.81806417657178</v>
+      </c>
+      <c r="BG36" s="1">
+        <v>6</v>
+      </c>
     </row>
-    <row r="37" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:59" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A37" s="208"/>
       <c r="B37" s="132">
         <v>5</v>
@@ -15943,8 +16178,14 @@
       <c r="AT37" s="232"/>
       <c r="AU37" s="193"/>
       <c r="AV37" s="194"/>
+      <c r="BF37" s="1">
+        <v>4.8958371788435597</v>
+      </c>
+      <c r="BG37" s="1">
+        <v>0.29136666442646852</v>
+      </c>
     </row>
-    <row r="38" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="198">
         <v>8</v>
       </c>
@@ -16073,7 +16314,7 @@
       </c>
       <c r="AV38" s="118"/>
     </row>
-    <row r="39" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="195"/>
       <c r="B39" s="130">
         <v>2</v>
@@ -16159,7 +16400,7 @@
       <c r="AT39" s="231"/>
       <c r="AV39" s="118"/>
     </row>
-    <row r="40" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="195"/>
       <c r="B40" s="130">
         <v>3</v>
@@ -16245,7 +16486,7 @@
       <c r="AT40" s="231"/>
       <c r="AV40" s="118"/>
     </row>
-    <row r="41" spans="1:48" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:59" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="207"/>
       <c r="B41" s="133">
         <v>4</v>
@@ -16331,7 +16572,7 @@
       <c r="AT41" s="231"/>
       <c r="AV41" s="118"/>
     </row>
-    <row r="42" spans="1:48" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:59" ht="16" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A42" s="208"/>
       <c r="B42" s="132">
         <v>5</v>
@@ -16416,7 +16657,7 @@
       <c r="AS42" s="241"/>
       <c r="AT42" s="232"/>
     </row>
-    <row r="44" spans="1:48" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:59" x14ac:dyDescent="0.2">
       <c r="G44" s="115"/>
     </row>
   </sheetData>

</xml_diff>